<commit_message>
food service program in bop
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -1905,7 +1905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D258"/>
+  <dimension ref="A1:D264"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6200,6 +6200,104 @@
       </c>
       <c r="D258" t="n">
         <v>100</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>YBBI</t>
+        </is>
+      </c>
+      <c r="B259" t="n">
+        <v>1</v>
+      </c>
+      <c r="C259" t="n">
+        <v>1</v>
+      </c>
+      <c r="D259" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>YBBI</t>
+        </is>
+      </c>
+      <c r="B260" t="n">
+        <v>2</v>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>SPO</t>
+        </is>
+      </c>
+      <c r="B261" t="n">
+        <v>1</v>
+      </c>
+      <c r="C261" t="n">
+        <v>1</v>
+      </c>
+      <c r="D261" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>SPO</t>
+        </is>
+      </c>
+      <c r="B262" t="n">
+        <v>2</v>
+      </c>
+      <c r="C262" t="n">
+        <v>2</v>
+      </c>
+      <c r="D262" t="n">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B263" t="n">
+        <v>2</v>
+      </c>
+      <c r="C263" t="n">
+        <v>2</v>
+      </c>
+      <c r="D263" t="n">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>VAL</t>
+        </is>
+      </c>
+      <c r="B264" t="n">
+        <v>1</v>
+      </c>
+      <c r="C264" t="n">
+        <v>1</v>
+      </c>
+      <c r="D264" t="n">
+        <v>185</v>
       </c>
     </row>
   </sheetData>
@@ -6213,7 +6311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E75"/>
+  <dimension ref="A1:E78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -7809,6 +7907,69 @@
         <v>4</v>
       </c>
       <c r="E75" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>YBBI</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>1</v>
+      </c>
+      <c r="C76" t="n">
+        <v>1</v>
+      </c>
+      <c r="D76" t="n">
+        <v>4</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>#,##0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>SPO</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>2</v>
+      </c>
+      <c r="C77" t="n">
+        <v>2</v>
+      </c>
+      <c r="D77" t="n">
+        <v>4</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>VAL</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>2</v>
+      </c>
+      <c r="C78" t="n">
+        <v>2</v>
+      </c>
+      <c r="D78" t="n">
+        <v>4</v>
+      </c>
+      <c r="E78" t="inlineStr">
         <is>
           <t>$#,##0.00</t>
         </is>

</xml_diff>

<commit_message>
major updates for formatting in all
</commit_message>
<xml_diff>
--- a/BOP/BOP Input File.xlsx
+++ b/BOP/BOP Input File.xlsx
@@ -2653,7 +2653,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D265"/>
+  <dimension ref="A1:D287"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -6657,7 +6657,7 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="242">
@@ -6691,7 +6691,7 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>125</v>
+        <v>110</v>
       </c>
     </row>
     <row r="244">
@@ -6703,10 +6703,8 @@
       <c r="B244" t="n">
         <v>1</v>
       </c>
-      <c r="C244" t="inlineStr">
-        <is>
-          <t>REST</t>
-        </is>
+      <c r="C244" t="n">
+        <v>1</v>
       </c>
       <c r="D244" t="n">
         <v>170</v>
@@ -7060,6 +7058,374 @@
       </c>
       <c r="D265" t="n">
         <v>185</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>FS_BR</t>
+        </is>
+      </c>
+      <c r="B266" t="n">
+        <v>1</v>
+      </c>
+      <c r="C266" t="n">
+        <v>1</v>
+      </c>
+      <c r="D266" t="n">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>FS_BR</t>
+        </is>
+      </c>
+      <c r="B267" t="n">
+        <v>2</v>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>FS_LS</t>
+        </is>
+      </c>
+      <c r="B268" t="n">
+        <v>1</v>
+      </c>
+      <c r="C268" t="n">
+        <v>2</v>
+      </c>
+      <c r="D268" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>FS_LS</t>
+        </is>
+      </c>
+      <c r="B269" t="n">
+        <v>3</v>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>FS_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B270" t="n">
+        <v>1</v>
+      </c>
+      <c r="C270" t="n">
+        <v>2</v>
+      </c>
+      <c r="D270" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>FS_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B271" t="n">
+        <v>3</v>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>FS_LL</t>
+        </is>
+      </c>
+      <c r="B272" t="n">
+        <v>1</v>
+      </c>
+      <c r="C272" t="n">
+        <v>1</v>
+      </c>
+      <c r="D272" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>FS_LL</t>
+        </is>
+      </c>
+      <c r="B273" t="n">
+        <v>2</v>
+      </c>
+      <c r="C273" t="n">
+        <v>2</v>
+      </c>
+      <c r="D273" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>W_LPGE</t>
+        </is>
+      </c>
+      <c r="B274" t="n">
+        <v>1</v>
+      </c>
+      <c r="C274" t="n">
+        <v>1</v>
+      </c>
+      <c r="D274" t="n">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>W_LPGE</t>
+        </is>
+      </c>
+      <c r="B275" t="n">
+        <v>2</v>
+      </c>
+      <c r="C275" t="n">
+        <v>2</v>
+      </c>
+      <c r="D275" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>O_LS</t>
+        </is>
+      </c>
+      <c r="B276" t="n">
+        <v>1</v>
+      </c>
+      <c r="C276" t="n">
+        <v>2</v>
+      </c>
+      <c r="D276" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>O_LS</t>
+        </is>
+      </c>
+      <c r="B277" t="n">
+        <v>3</v>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>O_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B278" t="n">
+        <v>1</v>
+      </c>
+      <c r="C278" t="n">
+        <v>2</v>
+      </c>
+      <c r="D278" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>O_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B279" t="n">
+        <v>3</v>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>O_DO</t>
+        </is>
+      </c>
+      <c r="B280" t="n">
+        <v>1</v>
+      </c>
+      <c r="C280" t="n">
+        <v>1</v>
+      </c>
+      <c r="D280" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>O_DO</t>
+        </is>
+      </c>
+      <c r="B281" t="n">
+        <v>4</v>
+      </c>
+      <c r="C281" t="n">
+        <v>4</v>
+      </c>
+      <c r="D281" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>O_DONM</t>
+        </is>
+      </c>
+      <c r="B282" t="n">
+        <v>1</v>
+      </c>
+      <c r="C282" t="n">
+        <v>1</v>
+      </c>
+      <c r="D282" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>FU</t>
+        </is>
+      </c>
+      <c r="B283" t="n">
+        <v>2</v>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>AS_LS</t>
+        </is>
+      </c>
+      <c r="B284" t="n">
+        <v>1</v>
+      </c>
+      <c r="C284" t="n">
+        <v>2</v>
+      </c>
+      <c r="D284" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>AS_LS</t>
+        </is>
+      </c>
+      <c r="B285" t="n">
+        <v>3</v>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>AS_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B286" t="n">
+        <v>1</v>
+      </c>
+      <c r="C286" t="n">
+        <v>2</v>
+      </c>
+      <c r="D286" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>AS_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B287" t="n">
+        <v>3</v>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -7073,7 +7439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E78"/>
+  <dimension ref="A1:E92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -8389,7 +8755,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>#,##0</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -8515,7 +8881,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>#,##0</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -8536,7 +8902,7 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>#,##0</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -8601,7 +8967,7 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>#,##0</t>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -8732,6 +9098,302 @@
       <c r="E78" t="inlineStr">
         <is>
           <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>FS_BR</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>REST</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>4</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>#,##0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>FS_LS</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>1</v>
+      </c>
+      <c r="C80" t="n">
+        <v>2</v>
+      </c>
+      <c r="D80" t="n">
+        <v>5</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>NoDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>FS_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>1</v>
+      </c>
+      <c r="C81" t="n">
+        <v>2</v>
+      </c>
+      <c r="D81" t="n">
+        <v>5</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>NoDecimal</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>FS_LL</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>1</v>
+      </c>
+      <c r="C82" t="n">
+        <v>1</v>
+      </c>
+      <c r="D82" t="n">
+        <v>4</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>W_LPGE</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>1</v>
+      </c>
+      <c r="C83" t="n">
+        <v>1</v>
+      </c>
+      <c r="D83" t="n">
+        <v>4</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>W_LPGE</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>2</v>
+      </c>
+      <c r="C84" t="n">
+        <v>2</v>
+      </c>
+      <c r="D84" t="n">
+        <v>4</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>O_LS</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>1</v>
+      </c>
+      <c r="C85" t="n">
+        <v>2</v>
+      </c>
+      <c r="D85" t="n">
+        <v>5</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>O_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>1</v>
+      </c>
+      <c r="C86" t="n">
+        <v>2</v>
+      </c>
+      <c r="D86" t="n">
+        <v>5</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>O_DO</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>2</v>
+      </c>
+      <c r="C87" t="n">
+        <v>2</v>
+      </c>
+      <c r="D87" t="n">
+        <v>4</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>O_DO</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>3</v>
+      </c>
+      <c r="C88" t="n">
+        <v>4</v>
+      </c>
+      <c r="D88" t="n">
+        <v>4</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>O_DONM</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>1</v>
+      </c>
+      <c r="C89" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" t="n">
+        <v>4</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>O_DONM</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>2</v>
+      </c>
+      <c r="C90" t="n">
+        <v>2</v>
+      </c>
+      <c r="D90" t="n">
+        <v>4</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>$#,##0.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>AS_LS</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>1</v>
+      </c>
+      <c r="C91" t="n">
+        <v>2</v>
+      </c>
+      <c r="D91" t="n">
+        <v>5</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>AS_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>1</v>
+      </c>
+      <c r="C92" t="n">
+        <v>2</v>
+      </c>
+      <c r="D92" t="n">
+        <v>5</v>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>$#,##0</t>
         </is>
       </c>
     </row>
@@ -8746,7 +9408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -9545,6 +10207,186 @@
         </is>
       </c>
       <c r="F25" t="inlineStr">
+        <is>
+          <t>C:REST</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>FS_LS</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>A:B</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Receipts Range</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>C:REST</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>FS_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>3</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>A:B</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Receipts Range</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>C:REST</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>O_LS</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>A:B</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Building plus Business Personal Property</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>C:REST</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>O_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>3</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>A:B</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Building plus Business Personal Property</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>C:REST</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>AS_LS</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A:B</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Receipts Range</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>C:REST</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>AS_LS_CURRENT</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>A:B</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Receipts Range</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
         <is>
           <t>C:REST</t>
         </is>
@@ -9614,7 +10456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -9864,10 +10706,94 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>CLBG</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>fit_width_repeat_header</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CLPP</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>fit_width_repeat_header</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>CLBI</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>fit_width_repeat_header</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CLGL</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>fit_width_repeat_header</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>CLEB</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>fit_width_repeat_header</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>RTRP</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>fit_width_repeat_header</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>LEAF</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>fit_width_repeat_header</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>*</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>fit_single_page</t>
         </is>

</xml_diff>